<commit_message>
Gobernanza por país: URLs específicas a documentos/anuncios (varias por celda)
- datos_gobernanza_detalle.py: se reemplazan las URLs de dominio por enlaces
  ESPECÍFICOS al documento/anuncio, con 2-3 fuentes por celda (148/190 celdas con
  >=2 URLs; 0 sin fuente). URLs localizadas vía búsqueda (jun-2026) y verificadas en
  resultados; oficiales (Diário da República RCM 2/2026, BOE RD 729/2023 y 817/2023,
  bundesregierung KI-Strategie PDF, BMAS Fortschreibung, bmftr Aktionsplan,
  Bundesnetzagentur, mddi.gov.sg, file.go.gov.sg/nais2023.pdf, regulations.ai) +
  anuncios (La Moncloa, digital.gob.es, portugal.gov.pt, observador) + secundarias.
- Regeneradas las 5 planillas por_pais/Gobernanza_<CC>_*.xlsx.

https://claude.ai/code/session_01MVDASqppDWTbc9vPCJJyhe
</commit_message>
<xml_diff>
--- a/data/paises_extra/por_pais/Gobernanza_DE_Alemania_ILIA2026.xlsx
+++ b/data/paises_extra/por_pais/Gobernanza_DE_Alemania_ILIA2026.xlsx
@@ -597,7 +597,9 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>https://www.ki-strategie-deutschland.de</t>
+          <t>https://www.bundesregierung.de/resource/blob/997532/1550276/3f7d3c41c6e05695741273e78b8039f2/2018-11-15-ki-strategie-data.pdf
+https://www.bmas.de/DE/Service/Presse/Pressemitteilungen/2020/kabinett-beschliesst-fortschreibung-der-ki-strategie-der-bundesregierung.html
+https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf</t>
         </is>
       </c>
     </row>
@@ -624,13 +626,13 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Documento vigente más reciente = Aktionsplan 2023 (base 2018/2020) → tramo 2022-23.  [confianza: ALTA]
-Nota matriz: EE: White Paper 2024-30 · SG: Update NAIS may-2026 = estrategia vigente (decisión operador) · DE: Aktionsplan 2023 · ES: Estrategia 2024 · PT: ANIA 2026-30</t>
+          <t>Documento vigente más reciente = Aktionsplan 2023 (base 2018/2020) → tramo 2022-23.  [confianza: ALTA]</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>https://www.bmftr.bund.de</t>
+          <t>https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf
+https://www.bmftr.bund.de/DE/Forschung/Schluesseltechnologien/KuenstlicheIntelligenz/KiAktionsplan/kiaktionsplan_node.html</t>
         </is>
       </c>
     </row>
@@ -662,7 +664,8 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>https://www.oecd.org</t>
+          <t>https://www.bmas.de/DE/Service/Presse/Pressemitteilungen/2020/kabinett-beschliesst-fortschreibung-der-ki-strategie-der-bundesregierung.html
+https://www.oecd.org/en/publications/oecd-artificial-intelligence-review-of-germany_609808d6-en.html</t>
         </is>
       </c>
     </row>
@@ -694,7 +697,8 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>https://www.oecd.org</t>
+          <t>https://www.oecd.org/en/publications/oecd-artificial-intelligence-review-of-germany_609808d6-en.html
+https://oecd.ai/en/wonk/review-germany-2024</t>
         </is>
       </c>
     </row>
@@ -721,13 +725,13 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>€5.000 millones hasta 2025 (Fortschreibung 2020).  [confianza: ALTA]
-Nota matriz: EE €85M · SG &gt;S$1.000M · DE €5.000M · ES €1.500M · PT &gt;€400M</t>
+          <t>€5.000 millones hasta 2025 (Fortschreibung 2020).  [confianza: ALTA]</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>https://www.ki-strategie-deutschland.de</t>
+          <t>https://www.bmas.de/DE/Service/Presse/Pressemitteilungen/2020/kabinett-beschliesst-fortschreibung-der-ki-strategie-der-bundesregierung.html
+https://www.ki-strategie-deutschland.de/</t>
         </is>
       </c>
     </row>
@@ -759,7 +763,8 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>https://www.bmftr.bund.de</t>
+          <t>https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf
+https://www.bmftr.bund.de/DE/Forschung/Schluesseltechnologien/KuenstlicheIntelligenz/KiAktionsplan/kiaktionsplan_node.html</t>
         </is>
       </c>
     </row>
@@ -791,7 +796,8 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>https://www.ki-strategie-deutschland.de</t>
+          <t>https://www.bundesregierung.de/resource/blob/997532/1550276/3f7d3c41c6e05695741273e78b8039f2/2018-11-15-ki-strategie-data.pdf
+https://www.plattform-lernende-systeme.de</t>
         </is>
       </c>
     </row>
@@ -823,7 +829,7 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>https://www.bmftr.bund.de</t>
+          <t>https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf</t>
         </is>
       </c>
     </row>
@@ -855,7 +861,8 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>https://knowledge4policy.ec.europa.eu</t>
+          <t>https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf
+https://www.ki-strategie-deutschland.de/</t>
         </is>
       </c>
     </row>
@@ -887,7 +894,8 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>https://www.ki-strategie-deutschland.de</t>
+          <t>https://www.ki-strategie-deutschland.de/
+https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf</t>
         </is>
       </c>
     </row>
@@ -919,7 +927,7 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>https://www.ki-strategie-deutschland.de</t>
+          <t>https://www.ki-strategie-deutschland.de/</t>
         </is>
       </c>
     </row>
@@ -951,7 +959,8 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>https://www.bmftr.bund.de</t>
+          <t>https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf
+https://www.ki-strategie-deutschland.de/</t>
         </is>
       </c>
     </row>
@@ -983,7 +992,8 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>https://www.bmftr.bund.de</t>
+          <t>https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf
+https://www.oecd.org/en/publications/oecd-artificial-intelligence-review-of-germany_609808d6-en.html</t>
         </is>
       </c>
     </row>
@@ -1010,12 +1020,13 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>'AI made in Europe'; Espacio Europeo de Investigación.  [confianza: MEDIA]</t>
+          <t>'AI made in Europe'; Espacio Europeo de Investigación; EU Coordinated Plan.  [confianza: MEDIA]</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>https://www.bmftr.bund.de</t>
+          <t>https://www.oecd.org/en/publications/progress-in-implementing-the-european-union-coordinated-plan-on-artificial-intelligence-volume-1_6d530a88-en/germany_f00f3020-en.html
+https://www.eubuero.de/de/akutelles-efr-2023-11-20-3499.html</t>
         </is>
       </c>
     </row>
@@ -1042,13 +1053,13 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Análisis externos: la estrategia 'apenas dio rol al género' → 0.  [confianza: MEDIA · PRELIM]
-Nota matriz: Solo ES recoge género (mención transversal); resto NO ENCONTRADO/0</t>
+          <t>Análisis externos: la estrategia 'apenas dio rol al género' → 0.  [confianza: MEDIA · PRELIM]</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>https://www.gleichstellungsbericht.de</t>
+          <t>https://www.gleichstellungsbericht.de
+https://www.bundesregierung.de/resource/blob/997532/1550276/3f7d3c41c6e05695741273e78b8039f2/2018-11-15-ki-strategie-data.pdf</t>
         </is>
       </c>
     </row>
@@ -1075,13 +1086,13 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>La Fortschreibung 2020 añade clima/medio ambiente. PRELIM.  [confianza: MEDIA · PRELIM]
-Nota matriz: PT: solo principio en EDN, no eje en ANIA</t>
+          <t>La Fortschreibung 2020 añade clima/medio ambiente. PRELIM.  [confianza: MEDIA · PRELIM]</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>https://www.ki-strategie-deutschland.de</t>
+          <t>https://www.bmas.de/DE/Service/Presse/Pressemitteilungen/2020/kabinett-beschliesst-fortschreibung-der-ki-strategie-der-bundesregierung.html
+https://www.ki-strategie-deutschland.de/</t>
         </is>
       </c>
     </row>
@@ -1108,13 +1119,12 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Consulta a asociaciones/talleres (2018); sin mecanismo ciudadano con resultados publicados → 2.  [confianza: MEDIA · PRELIM]
-Nota matriz: PT: consulta pública con resultados</t>
+          <t>Consulta a asociaciones/talleres (2018); sin mecanismo ciudadano con resultados publicados → 2.  [confianza: MEDIA · PRELIM]</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>https://www.bundesregierung.de</t>
+          <t>https://www.bundesregierung.de/resource/blob/997532/1550276/3f7d3c41c6e05695741273e78b8039f2/2018-11-15-ki-strategie-data.pdf</t>
         </is>
       </c>
     </row>
@@ -1141,13 +1151,13 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Elaboración: Gob (3 min.) + academia + industria + sociedad civil (PLS, ~200 expertos) (Gob+3).  [confianza: MEDIA · PRELIM]
-Nota matriz: PT: Gob+4</t>
+          <t>Elaboración: Gob (3 min.) + academia + industria + sociedad civil (PLS, ~200 expertos) (Gob+3).  [confianza: MEDIA · PRELIM]</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>https://www.plattform-lernende-systeme.de</t>
+          <t>https://www.plattform-lernende-systeme.de
+https://www.acatech.de/projekt/lernende-systeme-die-plattform-fuer-kuenstliche-intelligenz/</t>
         </is>
       </c>
     </row>
@@ -1179,7 +1189,8 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>https://en.acatech.de</t>
+          <t>https://www.acatech.de/projekt/lernende-systeme-die-plattform-fuer-kuenstliche-intelligenz/
+https://www.plattform-lernende-systeme.de</t>
         </is>
       </c>
     </row>
@@ -1206,13 +1217,14 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>&gt;1 institución: 3 ministerios líderes + PLS + Bundesnetzagentur (autoridad EU AI Act).  [confianza: ALTA]
-Nota matriz: ES: SEDIA+AESIA · DE: 3 min+PLS+BNetzA · PT: AMA+FCT+ANACOM</t>
+          <t>&gt;1 institución: 3 ministerios líderes + PLS + Bundesnetzagentur (autoridad EU AI Act).  [confianza: ALTA]</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>https://oecd.ai/en/dashboards/national/germany</t>
+          <t>https://www.oecd.org/en/publications/oecd-artificial-intelligence-review-of-germany_609808d6-en.html
+https://www.bundesnetzagentur.de/DE/Fachthemen/Digitales/KI/start_ki.html
+https://www.plattform-lernende-systeme.de</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1256,8 @@
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>https://www.oecd.org</t>
+          <t>https://www.oecd.org/en/publications/oecd-artificial-intelligence-review-of-germany_609808d6-en.html
+https://oecd.ai/en/wonk/review-germany-2024</t>
         </is>
       </c>
     </row>
@@ -1278,8 +1291,7 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>Participante (P-member, DIN) en SC 42.  [confianza: ALTA]
-Nota matriz: EE: no figura (verificar) · PT: Observador</t>
+          <t>Participante (P-member, DIN) en SC 42.  [confianza: ALTA]</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
@@ -1312,8 +1324,7 @@
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>Participante (P-member, DIN; secretaría) en SC 27.  [confianza: ALTA]
-Nota matriz: PT: Observador</t>
+          <t>Participante (P-member, DIN; secretaría) en SC 27.  [confianza: ALTA]</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
@@ -1345,14 +1356,14 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>OECD AI Principles + GPAI (fundador) + UNESCO + CoE (vía UE) + Plan UE = 2+.  [confianza: ALTA]
-Nota matriz: GPAI: miembros DE/ES; EE/SG/PT no individual</t>
+          <t>OECD AI Principles + GPAI (fundador) + UNESCO + CoE (vía UE) + Plan UE = 2+.  [confianza: ALTA]</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
           <t>https://oecd.ai/en/about/about-gpai
-https://oecd.ai/en/ai-principles</t>
+https://oecd.ai/en/ai-principles
+https://www.oecd.org/en/publications/progress-in-implementing-the-european-union-coordinated-plan-on-artificial-intelligence-volume-1_6d530a88-en/germany_f00f3020-en.html</t>
         </is>
       </c>
     </row>
@@ -1386,13 +1397,12 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>EU AI Act + ley nacional de implementación KI-MIG (borrador del Gabinete feb-2026).  [confianza: ALTA]
-Nota matriz: UE: EU AI Act (EE/DE/ES/PT). SG: soft law=1. ES/DE: además ley nacional</t>
+          <t>EU AI Act + ley nacional de implementación KI-MIG (borrador del Gabinete feb-2026).  [confianza: ALTA]</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>https://www.gleisslutz.com
+          <t>https://bmds.bund.de/service/gesetzgebungsverfahren/gesetz-zur-durchfuehrung-der-ki-verordnung
 https://eur-lex.europa.eu/eli/reg/2024/1689/oj</t>
         </is>
       </c>
@@ -1452,13 +1462,13 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Bundesnetzagentur: sandbox + AI Service Desk (2025-26).  [confianza: ALTA]
-Nota matriz: ES: 1er sandbox UE</t>
+          <t>Bundesnetzagentur: KI-Reallabore (sandbox) + AI Service Desk (2025-26).  [confianza: ALTA]</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>https://www.bundesnetzagentur.de</t>
+          <t>https://www.bundesnetzagentur.de/DE/Fachthemen/Digitales/KI/5_Innovationen/start.html
+https://www.bundesnetzagentur.de/DE/Fachthemen/Digitales/KI/start_ki.html</t>
         </is>
       </c>
     </row>
@@ -1518,8 +1528,7 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>BfDI + 16 autoridades de los Länder.  [confianza: ALTA]
-Nota matriz: AKI/PDPC/BfDI/AEPD/CNPD</t>
+          <t>BfDI + 16 autoridades de los Länder.  [confianza: ALTA]</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -1558,8 +1567,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>NO ENCONTRADO por pilar; GCI 2024 = Tier 1 (total ~97,85). Pilares solo en anexo PDF.  [confianza: MANUAL]
-Nota matriz: Solo ES con pilares; resto Tier 1, pilares en anexo PDF</t>
+          <t>NO ENCONTRADO por pilar; GCI 2024 = Tier 1 (total ~97,85). Pilares solo en anexo PDF.  [confianza: MANUAL]</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
@@ -1724,8 +1732,7 @@
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>NO ENCONTRADO; DE cubierto por GIRAI; puntaje por área en portal JS/PDF.  [confianza: MANUAL]
-Nota matriz: Portal JS/PDF → extracción manual</t>
+          <t>NO ENCONTRADO; DE cubierto por GIRAI; puntaje por área en portal JS/PDF.  [confianza: MANUAL]</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
@@ -1757,8 +1764,7 @@
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>NO ENCONTRADO (portal JS/PDF).  [confianza: MANUAL]
-Nota matriz: Idem</t>
+          <t>NO ENCONTRADO (portal JS/PDF).  [confianza: MANUAL]</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
@@ -1790,8 +1796,7 @@
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>86,44 en 'Affordable &amp; clean energy', NRI ed. 2025.  [confianza: MEDIA-ALTA]
-Nota matriz: ES: ver página país NRI</t>
+          <t>86,44 en 'Affordable &amp; clean energy', NRI ed. 2025.  [confianza: MEDIA-ALTA]</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
@@ -1823,8 +1828,7 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>58,64 % (2024) / 59,09 % (2025) renovable total. Excl. toda hidro 53,84 %; hidro 4,81 %. (ERNC excl. gran hidro: efecto menor.)  [confianza: ALTA]
-Nota matriz: 2024, renovables total. ES/PT/DE: ERNC excl. gran hidro es menor (ver energia_*.md)</t>
+          <t>58,64 % (2024) / 59,09 % (2025) renovable total. Excl. toda hidro 53,84 %; hidro 4,81 %. (ERNC excl. gran hidro: efecto menor.)  [confianza: ALTA]</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Gobernanza por país: tipado oficial/secundaria + ≥2 fuentes en todas las celdas
- generar_gobernanza_por_pais.py: cada URL se etiqueta [oficial] (gobierno, BOE/
  Diário da República, ISO/ITU, OCDE, dato primario) o [secundaria] (prensa, despacho,
  agregador); las oficiales se listan primero. Cabecera y leyenda actualizadas.
- datos_gobernanza_detalle.py: bloque de segundas fuentes verificadas para que ninguna
  celda quede con una sola URL (190/190 con ≥2): ISO SC27 (espejo), GIRAI edición
  corregida + Global Center, DLA Piper (autoridad) por país, AI Act sandbox/ref,
  2ª referencia de estrategia, y PDF-país NRI 2025 (spain/estonia/singapore.pdf) o
  informe completo nri-2025.pdf. Solo URLs vistas en resultados/compendio.
- Regeneradas las 5 planillas.

https://claude.ai/code/session_01MVDASqppDWTbc9vPCJJyhe
</commit_message>
<xml_diff>
--- a/data/paises_extra/por_pais/Gobernanza_DE_Alemania_ILIA2026.xlsx
+++ b/data/paises_extra/por_pais/Gobernanza_DE_Alemania_ILIA2026.xlsx
@@ -525,7 +525,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Compendio exhaustivo de URLs: gobernanza/FUENTES_gobernanza_EE_SG.md (EE/SG) · gobernanza_&lt;país&gt;.md, gobernanza_estandares_*.md, etica_seguridad_*.md, energia_*.md (DE/ES/PT). Rúbricas: gobernanza/RUBRICAS_gobernanza.md.</t>
+          <t>Cada URL va etiquetada [oficial] (gobierno, BOE/Diário da República, ISO/ITU, OCDE, dato primario) o [secundaria] (prensa, despacho, agregador). Compendio exhaustivo: gobernanza/FUENTES_gobernanza_EE_SG.md (EE/SG) · gobernanza_&lt;país&gt;.md, gobernanza_estandares_*.md, etica_seguridad_*.md, energia_*.md (DE/ES/PT). Rúbricas: gobernanza/RUBRICAS_gobernanza.md.</t>
         </is>
       </c>
     </row>
@@ -558,7 +558,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Fuentes y URLs</t>
+          <t>Fuentes y URLs  ([oficial] primaria · [secundaria] corrobora)</t>
         </is>
       </c>
     </row>
@@ -597,9 +597,9 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>https://www.bundesregierung.de/resource/blob/997532/1550276/3f7d3c41c6e05695741273e78b8039f2/2018-11-15-ki-strategie-data.pdf
-https://www.bmas.de/DE/Service/Presse/Pressemitteilungen/2020/kabinett-beschliesst-fortschreibung-der-ki-strategie-der-bundesregierung.html
-https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf</t>
+          <t>[oficial] https://www.bundesregierung.de/resource/blob/997532/1550276/3f7d3c41c6e05695741273e78b8039f2/2018-11-15-ki-strategie-data.pdf
+[oficial] https://www.bmas.de/DE/Service/Presse/Pressemitteilungen/2020/kabinett-beschliesst-fortschreibung-der-ki-strategie-der-bundesregierung.html
+[oficial] https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf</t>
         </is>
       </c>
     </row>
@@ -631,8 +631,8 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf
-https://www.bmftr.bund.de/DE/Forschung/Schluesseltechnologien/KuenstlicheIntelligenz/KiAktionsplan/kiaktionsplan_node.html</t>
+          <t>[oficial] https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf
+[oficial] https://www.bmftr.bund.de/DE/Forschung/Schluesseltechnologien/KuenstlicheIntelligenz/KiAktionsplan/kiaktionsplan_node.html</t>
         </is>
       </c>
     </row>
@@ -664,8 +664,8 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>https://www.bmas.de/DE/Service/Presse/Pressemitteilungen/2020/kabinett-beschliesst-fortschreibung-der-ki-strategie-der-bundesregierung.html
-https://www.oecd.org/en/publications/oecd-artificial-intelligence-review-of-germany_609808d6-en.html</t>
+          <t>[oficial] https://www.bmas.de/DE/Service/Presse/Pressemitteilungen/2020/kabinett-beschliesst-fortschreibung-der-ki-strategie-der-bundesregierung.html
+[oficial] https://www.oecd.org/en/publications/oecd-artificial-intelligence-review-of-germany_609808d6-en.html</t>
         </is>
       </c>
     </row>
@@ -697,8 +697,8 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>https://www.oecd.org/en/publications/oecd-artificial-intelligence-review-of-germany_609808d6-en.html
-https://oecd.ai/en/wonk/review-germany-2024</t>
+          <t>[oficial] https://www.oecd.org/en/publications/oecd-artificial-intelligence-review-of-germany_609808d6-en.html
+[oficial] https://oecd.ai/en/wonk/review-germany-2024</t>
         </is>
       </c>
     </row>
@@ -730,8 +730,8 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>https://www.bmas.de/DE/Service/Presse/Pressemitteilungen/2020/kabinett-beschliesst-fortschreibung-der-ki-strategie-der-bundesregierung.html
-https://www.ki-strategie-deutschland.de/</t>
+          <t>[oficial] https://www.bmas.de/DE/Service/Presse/Pressemitteilungen/2020/kabinett-beschliesst-fortschreibung-der-ki-strategie-der-bundesregierung.html
+[oficial] https://www.ki-strategie-deutschland.de/</t>
         </is>
       </c>
     </row>
@@ -763,8 +763,8 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf
-https://www.bmftr.bund.de/DE/Forschung/Schluesseltechnologien/KuenstlicheIntelligenz/KiAktionsplan/kiaktionsplan_node.html</t>
+          <t>[oficial] https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf
+[oficial] https://www.bmftr.bund.de/DE/Forschung/Schluesseltechnologien/KuenstlicheIntelligenz/KiAktionsplan/kiaktionsplan_node.html</t>
         </is>
       </c>
     </row>
@@ -796,8 +796,8 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>https://www.bundesregierung.de/resource/blob/997532/1550276/3f7d3c41c6e05695741273e78b8039f2/2018-11-15-ki-strategie-data.pdf
-https://www.plattform-lernende-systeme.de</t>
+          <t>[oficial] https://www.bundesregierung.de/resource/blob/997532/1550276/3f7d3c41c6e05695741273e78b8039f2/2018-11-15-ki-strategie-data.pdf
+[oficial] https://www.plattform-lernende-systeme.de</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,8 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf</t>
+          <t>[oficial] https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf
+[oficial] https://www.ki-strategie-deutschland.de/</t>
         </is>
       </c>
     </row>
@@ -861,8 +862,8 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf
-https://www.ki-strategie-deutschland.de/</t>
+          <t>[oficial] https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf
+[oficial] https://www.ki-strategie-deutschland.de/</t>
         </is>
       </c>
     </row>
@@ -894,8 +895,8 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>https://www.ki-strategie-deutschland.de/
-https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf</t>
+          <t>[oficial] https://www.ki-strategie-deutschland.de/
+[oficial] https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf</t>
         </is>
       </c>
     </row>
@@ -927,7 +928,8 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>https://www.ki-strategie-deutschland.de/</t>
+          <t>[oficial] https://www.ki-strategie-deutschland.de/
+[oficial] https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf</t>
         </is>
       </c>
     </row>
@@ -959,8 +961,8 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf
-https://www.ki-strategie-deutschland.de/</t>
+          <t>[oficial] https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf
+[oficial] https://www.ki-strategie-deutschland.de/</t>
         </is>
       </c>
     </row>
@@ -992,8 +994,8 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf
-https://www.oecd.org/en/publications/oecd-artificial-intelligence-review-of-germany_609808d6-en.html</t>
+          <t>[oficial] https://www.ki-strategie-deutschland.de/files/downloads/Aktionsplan_Kuenstliche_Intelligenz_2023.pdf
+[oficial] https://www.oecd.org/en/publications/oecd-artificial-intelligence-review-of-germany_609808d6-en.html</t>
         </is>
       </c>
     </row>
@@ -1025,8 +1027,8 @@
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>https://www.oecd.org/en/publications/progress-in-implementing-the-european-union-coordinated-plan-on-artificial-intelligence-volume-1_6d530a88-en/germany_f00f3020-en.html
-https://www.eubuero.de/de/akutelles-efr-2023-11-20-3499.html</t>
+          <t>[oficial] https://www.oecd.org/en/publications/progress-in-implementing-the-european-union-coordinated-plan-on-artificial-intelligence-volume-1_6d530a88-en/germany_f00f3020-en.html
+[secundaria] https://www.eubuero.de/de/akutelles-efr-2023-11-20-3499.html</t>
         </is>
       </c>
     </row>
@@ -1058,8 +1060,8 @@
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>https://www.gleichstellungsbericht.de
-https://www.bundesregierung.de/resource/blob/997532/1550276/3f7d3c41c6e05695741273e78b8039f2/2018-11-15-ki-strategie-data.pdf</t>
+          <t>[oficial] https://www.bundesregierung.de/resource/blob/997532/1550276/3f7d3c41c6e05695741273e78b8039f2/2018-11-15-ki-strategie-data.pdf
+[secundaria] https://www.gleichstellungsbericht.de</t>
         </is>
       </c>
     </row>
@@ -1091,8 +1093,8 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>https://www.bmas.de/DE/Service/Presse/Pressemitteilungen/2020/kabinett-beschliesst-fortschreibung-der-ki-strategie-der-bundesregierung.html
-https://www.ki-strategie-deutschland.de/</t>
+          <t>[oficial] https://www.bmas.de/DE/Service/Presse/Pressemitteilungen/2020/kabinett-beschliesst-fortschreibung-der-ki-strategie-der-bundesregierung.html
+[oficial] https://www.ki-strategie-deutschland.de/</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1126,8 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>https://www.bundesregierung.de/resource/blob/997532/1550276/3f7d3c41c6e05695741273e78b8039f2/2018-11-15-ki-strategie-data.pdf</t>
+          <t>[oficial] https://www.bundesregierung.de/resource/blob/997532/1550276/3f7d3c41c6e05695741273e78b8039f2/2018-11-15-ki-strategie-data.pdf
+[oficial] https://www.ki-strategie-deutschland.de/</t>
         </is>
       </c>
     </row>
@@ -1156,8 +1159,8 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>https://www.plattform-lernende-systeme.de
-https://www.acatech.de/projekt/lernende-systeme-die-plattform-fuer-kuenstliche-intelligenz/</t>
+          <t>[oficial] https://www.plattform-lernende-systeme.de
+[oficial] https://www.acatech.de/projekt/lernende-systeme-die-plattform-fuer-kuenstliche-intelligenz/</t>
         </is>
       </c>
     </row>
@@ -1189,8 +1192,8 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>https://www.acatech.de/projekt/lernende-systeme-die-plattform-fuer-kuenstliche-intelligenz/
-https://www.plattform-lernende-systeme.de</t>
+          <t>[oficial] https://www.acatech.de/projekt/lernende-systeme-die-plattform-fuer-kuenstliche-intelligenz/
+[oficial] https://www.plattform-lernende-systeme.de</t>
         </is>
       </c>
     </row>
@@ -1222,9 +1225,9 @@
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>https://www.oecd.org/en/publications/oecd-artificial-intelligence-review-of-germany_609808d6-en.html
-https://www.bundesnetzagentur.de/DE/Fachthemen/Digitales/KI/start_ki.html
-https://www.plattform-lernende-systeme.de</t>
+          <t>[oficial] https://www.oecd.org/en/publications/oecd-artificial-intelligence-review-of-germany_609808d6-en.html
+[oficial] https://www.bundesnetzagentur.de/DE/Fachthemen/Digitales/KI/start_ki.html
+[oficial] https://www.plattform-lernende-systeme.de</t>
         </is>
       </c>
     </row>
@@ -1256,8 +1259,8 @@
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>https://www.oecd.org/en/publications/oecd-artificial-intelligence-review-of-germany_609808d6-en.html
-https://oecd.ai/en/wonk/review-germany-2024</t>
+          <t>[oficial] https://www.oecd.org/en/publications/oecd-artificial-intelligence-review-of-germany_609808d6-en.html
+[oficial] https://oecd.ai/en/wonk/review-germany-2024</t>
         </is>
       </c>
     </row>
@@ -1296,8 +1299,8 @@
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>https://www.iso.org/committee/6794475.html?view=participation
-https://jtc1info.org/sd-2-history/jtc1-subcommittees/sc-42/</t>
+          <t>[oficial] https://www.iso.org/committee/6794475.html?view=participation
+[secundaria] https://jtc1info.org/sd-2-history/jtc1-subcommittees/sc-42/</t>
         </is>
       </c>
     </row>
@@ -1329,7 +1332,8 @@
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>https://www.iso.org/committee/45306.html?view=participation</t>
+          <t>[oficial] https://www.iso.org/committee/45306.html?view=participation
+[secundaria] https://en.wikipedia.org/wiki/ISO/IEC_JTC_1/SC_27</t>
         </is>
       </c>
     </row>
@@ -1361,9 +1365,9 @@
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>https://oecd.ai/en/about/about-gpai
-https://oecd.ai/en/ai-principles
-https://www.oecd.org/en/publications/progress-in-implementing-the-european-union-coordinated-plan-on-artificial-intelligence-volume-1_6d530a88-en/germany_f00f3020-en.html</t>
+          <t>[oficial] https://oecd.ai/en/about/about-gpai
+[oficial] https://oecd.ai/en/ai-principles
+[oficial] https://www.oecd.org/en/publications/progress-in-implementing-the-european-union-coordinated-plan-on-artificial-intelligence-volume-1_6d530a88-en/germany_f00f3020-en.html</t>
         </is>
       </c>
     </row>
@@ -1402,8 +1406,8 @@
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>https://bmds.bund.de/service/gesetzgebungsverfahren/gesetz-zur-durchfuehrung-der-ki-verordnung
-https://eur-lex.europa.eu/eli/reg/2024/1689/oj</t>
+          <t>[oficial] https://bmds.bund.de/service/gesetzgebungsverfahren/gesetz-zur-durchfuehrung-der-ki-verordnung
+[oficial] https://eur-lex.europa.eu/eli/reg/2024/1689/oj</t>
         </is>
       </c>
     </row>
@@ -1435,7 +1439,8 @@
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>https://eur-lex.europa.eu/eli/reg/2024/1689/oj</t>
+          <t>[oficial] https://eur-lex.europa.eu/eli/reg/2024/1689/oj
+[secundaria] https://artificialintelligenceact.eu</t>
         </is>
       </c>
     </row>
@@ -1467,8 +1472,8 @@
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>https://www.bundesnetzagentur.de/DE/Fachthemen/Digitales/KI/5_Innovationen/start.html
-https://www.bundesnetzagentur.de/DE/Fachthemen/Digitales/KI/start_ki.html</t>
+          <t>[oficial] https://www.bundesnetzagentur.de/DE/Fachthemen/Digitales/KI/5_Innovationen/start.html
+[oficial] https://www.bundesnetzagentur.de/DE/Fachthemen/Digitales/KI/start_ki.html</t>
         </is>
       </c>
     </row>
@@ -1500,8 +1505,8 @@
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>https://www.dlapiperdataprotection.com/?t=law&amp;c=DE
-https://www.bfdi.bund.de</t>
+          <t>[oficial] https://www.bfdi.bund.de
+[secundaria] https://www.dlapiperdataprotection.com/?t=law&amp;c=DE</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1538,8 @@
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>https://www.bfdi.bund.de</t>
+          <t>[oficial] https://www.bfdi.bund.de
+[secundaria] https://www.dlapiperdataprotection.com/?t=authority&amp;c=DE</t>
         </is>
       </c>
     </row>
@@ -1572,8 +1578,8 @@
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>https://www.itu.int/epublications/publication/global-cybersecurity-index-2024
-https://data360.worldbank.org/en/indicator/ITU_GCI_GCI_OVRL_SCRE</t>
+          <t>[oficial] https://www.itu.int/epublications/publication/global-cybersecurity-index-2024
+[oficial] https://data360.worldbank.org/en/indicator/ITU_GCI_GCI_OVRL_SCRE</t>
         </is>
       </c>
     </row>
@@ -1605,8 +1611,8 @@
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>https://www.itu.int/epublications/publication/global-cybersecurity-index-2024
-https://data360.worldbank.org/en/indicator/ITU_GCI_GCI_OVRL_SCRE</t>
+          <t>[oficial] https://www.itu.int/epublications/publication/global-cybersecurity-index-2024
+[oficial] https://data360.worldbank.org/en/indicator/ITU_GCI_GCI_OVRL_SCRE</t>
         </is>
       </c>
     </row>
@@ -1638,8 +1644,8 @@
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>https://www.itu.int/epublications/publication/global-cybersecurity-index-2024
-https://data360.worldbank.org/en/indicator/ITU_GCI_GCI_OVRL_SCRE</t>
+          <t>[oficial] https://www.itu.int/epublications/publication/global-cybersecurity-index-2024
+[oficial] https://data360.worldbank.org/en/indicator/ITU_GCI_GCI_OVRL_SCRE</t>
         </is>
       </c>
     </row>
@@ -1671,8 +1677,8 @@
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>https://www.itu.int/epublications/publication/global-cybersecurity-index-2024
-https://data360.worldbank.org/en/indicator/ITU_GCI_GCI_OVRL_SCRE</t>
+          <t>[oficial] https://www.itu.int/epublications/publication/global-cybersecurity-index-2024
+[oficial] https://data360.worldbank.org/en/indicator/ITU_GCI_GCI_OVRL_SCRE</t>
         </is>
       </c>
     </row>
@@ -1704,8 +1710,8 @@
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>https://www.itu.int/epublications/publication/global-cybersecurity-index-2024
-https://data360.worldbank.org/en/indicator/ITU_GCI_GCI_OVRL_SCRE</t>
+          <t>[oficial] https://www.itu.int/epublications/publication/global-cybersecurity-index-2024
+[oficial] https://data360.worldbank.org/en/indicator/ITU_GCI_GCI_OVRL_SCRE</t>
         </is>
       </c>
     </row>
@@ -1737,7 +1743,8 @@
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>https://www.global-index.ai</t>
+          <t>[oficial] https://www.global-index.ai
+[secundaria] https://girai-report-2024-corrected-edition.tiiny.site/</t>
         </is>
       </c>
     </row>
@@ -1769,7 +1776,8 @@
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>https://www.global-index.ai</t>
+          <t>[oficial] https://www.global-index.ai
+[oficial] https://www.globalcenter.ai/</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1809,8 @@
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>https://networkreadinessindex.org/country/germany/</t>
+          <t>[oficial] https://networkreadinessindex.org/country/germany/
+[oficial] https://download.networkreadinessindex.org/reports/data/2025/nri-2025.pdf</t>
         </is>
       </c>
     </row>
@@ -1833,8 +1842,8 @@
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/owid/energy-data/master/owid-energy-data.csv
-https://ember-energy.org/data/electricity-data-explorer/</t>
+          <t>[oficial] https://raw.githubusercontent.com/owid/energy-data/master/owid-energy-data.csv
+[oficial] https://ember-energy.org/data/electricity-data-explorer/</t>
         </is>
       </c>
     </row>

</xml_diff>